<commit_message>
Customer version of Almotasem RFQ: final prices only
Removes list prices, discount and price-list references; options show
their final price and are included in Unit Price.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u8mjeREzpMeGcR4rGo8uz
</commit_message>
<xml_diff>
--- a/gearbox-selection/Almotasem_Gearboxes_RFQ_450_Units.xlsx
+++ b/gearbox-selection/Almotasem_Gearboxes_RFQ_450_Units.xlsx
@@ -1580,7 +1580,7 @@
     <row r="4">
       <c r="A4" s="169" t="inlineStr">
         <is>
-          <t>Supplier offer: İ.Mak (Turkey) equivalents · EUR, EXW · net after 35% discount on İ.Mak price list 26.01.2026 · Unit Price includes all quoted options</t>
+          <t>Offer: İ.Mak (Turkey) equivalent units · Prices in EUR, EXW · Unit Price is the final price per unit, including the options listed in the Notes column</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="N7" s="172" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="N8" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="N9" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="N10" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="N11" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="N12" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="N13" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="N14" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø18 | Options (list → net): Output flange €7.00 → €4.55; Torque arm €9.00 → €5.85; Output shaft €8.00 → €5.20</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 40 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø18 | Options included in Unit Price: Output flange €4.55; Torque arm €5.85; Output shaft €5.20</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="N15" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="N16" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="N17" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2396,7 +2396,7 @@
       </c>
       <c r="N18" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="N19" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="N20" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="N21" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="N22" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø25 | Options (list → net): Output flange €8.00 → €5.20; Torque arm €11.00 → €7.15; Output shaft €9.00 → €5.85</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 50 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø25 | Options included in Unit Price: Output flange €5.20; Torque arm €7.15; Output shaft €5.85</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="N23" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="N24" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -2830,7 +2830,7 @@
       </c>
       <c r="N25" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="N26" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="N27" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="N28" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="N29" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="N30" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø25 | Options (list → net): Output flange €10.00 → €6.50; Torque arm €15.00 → €9.75; Output shaft €11.00 → €7.15</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 63 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø25 | Options included in Unit Price: Output flange €6.50; Torque arm €9.75; Output shaft €7.15</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="N31" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3264,7 +3264,7 @@
       </c>
       <c r="N32" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="N33" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="N34" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="N35" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="N36" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="N37" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="N38" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø28 | Options (list → net): Output flange €15.00 → €9.75; Torque arm €25.00 → €16.25; Output shaft €15.00 → €9.75</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 75 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø28 | Options included in Unit Price: Output flange €9.75; Torque arm €16.25; Output shaft €9.75</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="N39" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="N40" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=15 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=15, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="N41" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="N42" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=25 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=25, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="N43" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="N44" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="N45" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="N46" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø35 | Options (list → net): Output flange €23.00 → €14.95; Torque arm €40.00 → €26.00; Output shaft €24.00 → €15.60</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 90 i=60 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=60, hollow Ø35 | Options included in Unit Price: Output flange €14.95; Torque arm €26.00; Output shaft €15.60</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="N47" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø42 | Options (list → net): Output flange €35.00 → €22.75; Torque arm €67.00 → €43.55; Output shaft €39.00 → €25.35</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=10 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=10, hollow Ø42 | Options included in Unit Price: Output flange €22.75; Torque arm €43.55; Output shaft €25.35</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="N48" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø42 | Options (list → net): Output flange €35.00 → €22.75; Torque arm €67.00 → €43.55; Output shaft €39.00 → €25.35</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=20 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=20, hollow Ø42 | Options included in Unit Price: Output flange €22.75; Torque arm €43.55; Output shaft €25.35</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="N49" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø42 | Options (list → net): Output flange €35.00 → €22.75; Torque arm €67.00 → €43.55; Output shaft €39.00 → €25.35</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=30 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=30, hollow Ø42 | Options included in Unit Price: Output flange €22.75; Torque arm €43.55; Output shaft €25.35</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="N50" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø42 | Options (list → net): Output flange €35.00 → €22.75; Torque arm €67.00 → €43.55; Output shaft €39.00 → €25.35</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=40 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=40, hollow Ø42 | Options included in Unit Price: Output flange €22.75; Torque arm €43.55; Output shaft €25.35</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="N51" s="175" t="inlineStr">
         <is>
-          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø42 | Options (list → net): Output flange €35.00 → €22.75; Torque arm €67.00 → €43.55; Output shaft €39.00 → €25.35</t>
+          <t>Factory-filled oil; quote output flange, torque arm and shafts separately || OFFERED: İ.Mak SP 110 i=50 (IEC B14/B5 input flange, hollow output) | Direct NMRV equivalent, i=50, hollow Ø42 | Options included in Unit Price: Output flange €22.75; Torque arm €43.55; Output shaft €25.35</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="N52" s="175" t="inlineStr">
         <is>
-          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=52 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:52 instead of 1:50; hollow Ø50 (NMRV130 = Ø45) | Options (list → net): Output flange €60.00 → €39.00; Torque arm €45.00 → €29.25; Output shaft €34.00 → €22.10</t>
+          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=52 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:52 instead of 1:50; hollow Ø50 (NMRV130 = Ø45) | Options included in Unit Price: Output flange €39.00; Torque arm €29.25; Output shaft €22.10</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="N53" s="175" t="inlineStr">
         <is>
-          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=65 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:65 instead of 1:60; hollow Ø50 (NMRV130 = Ø45) | Options (list → net): Output flange €60.00 → €39.00; Torque arm €45.00 → €29.25; Output shaft €34.00 → €22.10</t>
+          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=65 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:65 instead of 1:60; hollow Ø50 (NMRV130 = Ø45) | Options included in Unit Price: Output flange €39.00; Torque arm €29.25; Output shaft €22.10</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="N54" s="175" t="inlineStr">
         <is>
-          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=52 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:52 instead of 1:50; hollow Ø50 | Options (list → net): Output flange €60.00 → €39.00; Torque arm €45.00 → €29.25; Output shaft €34.00 → €22.10</t>
+          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=52 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:52 instead of 1:50; hollow Ø50 | Options included in Unit Price: Output flange €39.00; Torque arm €29.25; Output shaft €22.10</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="N55" s="175" t="inlineStr">
         <is>
-          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=65 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:65 instead of 1:60; hollow Ø50 | Options (list → net): Output flange €60.00 → €39.00; Torque arm €45.00 → €29.25; Output shaft €34.00 → €22.10</t>
+          <t>Cast-iron housing required; factory-filled oil || OFFERED: İ.Mak İRSAP 127 i=65 (IEC B14/B5 input flange, hollow output) | Cast-iron İRSA 127 offered (S series is aluminium); ratio 1:65 instead of 1:60; hollow Ø50 | Options included in Unit Price: Output flange €39.00; Torque arm €29.25; Output shaft €22.10</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="N56" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 42 i=9.845 + IEC 71 B5 input (code 155) | Catalogue ratio i=9.845 (n2≈142 rpm), Sf 1.94 at 0.37 kW; Gearmotor alternative: İRAM 42 / 71 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 42 i=9.845 + IEC 71 B5 input (code 155) | Catalogue ratio i=9.845 (n2≈142 rpm), Sf 1.94 at 0.37 kW; Gearmotor alternative: İRAM 42 / 71 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="N57" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 43 i=20.0 + IEC 71 B5 input (code 155) | Catalogue ratio i=20.0 (n2≈69 rpm), Sf 1.68 at 0.37 kW; Gearmotor alternative: İRAM 43 / 71 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 43 i=20.0 + IEC 71 B5 input (code 155) | Catalogue ratio i=20.0 (n2≈69 rpm), Sf 1.68 at 0.37 kW; Gearmotor alternative: İRAM 43 / 71 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -4882,7 +4882,7 @@
       </c>
       <c r="N58" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=31.33 + IEC 71 B5 input (code 155) | Catalogue ratio i=31.33 (n2≈44 rpm), Sf 2.49 at 0.37 kW; Gearmotor alternative: İRAM 53 / 71 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=31.33 + IEC 71 B5 input (code 155) | Catalogue ratio i=31.33 (n2≈44 rpm), Sf 2.49 at 0.37 kW; Gearmotor alternative: İRAM 53 / 71 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -4946,7 +4946,7 @@
       </c>
       <c r="N59" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=39.09 + IEC 71 B5 input (code 155) | Catalogue ratio i=39.09 (n2≈35 rpm), Sf 2.07 at 0.37 kW; Gearmotor alternative: İRAM 53 / 71 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=39.09 + IEC 71 B5 input (code 155) | Catalogue ratio i=39.09 (n2≈35 rpm), Sf 2.07 at 0.37 kW; Gearmotor alternative: İRAM 53 / 71 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="N60" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 52 i=9.47 + IEC 80 B5 input (code 155) | Catalogue ratio i=9.47 (n2≈147 rpm), Sf 4.4 at 0.55 kW; Gearmotor alternative: İRAM 52 / 80 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 52 i=9.47 + IEC 80 B5 input (code 155) | Catalogue ratio i=9.47 (n2≈147 rpm), Sf 4.4 at 0.55 kW; Gearmotor alternative: İRAM 52 / 80 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5074,7 +5074,7 @@
       </c>
       <c r="N61" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 43 i=14.6 + IEC 80 B5 input (code 155) | Catalogue ratio i=14.6 (n2≈95 rpm), Sf 1.54 at 0.55 kW; Gearmotor alternative: İRAM 43 / 80 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 43 i=14.6 + IEC 80 B5 input (code 155) | Catalogue ratio i=14.6 (n2≈95 rpm), Sf 1.54 at 0.55 kW; Gearmotor alternative: İRAM 43 / 80 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="N62" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=21.88 + IEC 80 B5 input (code 155) | Catalogue ratio i=21.88 (n2≈63 rpm), Sf 2.22 at 0.55 kW; Gearmotor alternative: İRAM 53 / 80 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=21.88 + IEC 80 B5 input (code 155) | Catalogue ratio i=21.88 (n2≈63 rpm), Sf 2.22 at 0.55 kW; Gearmotor alternative: İRAM 53 / 80 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="N63" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=31.33 + IEC 80 B5 input (code 155) | Catalogue ratio i=31.33 (n2≈44 rpm), Sf 1.68 at 0.55 kW; Gearmotor alternative: İRAM 53 / 80 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=31.33 + IEC 80 B5 input (code 155) | Catalogue ratio i=31.33 (n2≈44 rpm), Sf 1.68 at 0.55 kW; Gearmotor alternative: İRAM 53 / 80 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="N64" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 52 i=9.47 + IEC 80 B5 input (code 155) | Catalogue ratio i=9.47 (n2≈147 rpm), Sf 3.23 at 0.75 kW; Gearmotor alternative: İRAM 52 / 80 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 52 i=9.47 + IEC 80 B5 input (code 155) | Catalogue ratio i=9.47 (n2≈147 rpm), Sf 3.23 at 0.75 kW; Gearmotor alternative: İRAM 52 / 80 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="N65" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=19.69 + IEC 80 B5 input (code 155) | Catalogue ratio i=19.69 (n2≈71 rpm), Sf 1.81 at 0.75 kW; Gearmotor alternative: İRAM 53 / 80 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 53 i=19.69 + IEC 80 B5 input (code 155) | Catalogue ratio i=19.69 (n2≈71 rpm), Sf 1.81 at 0.75 kW; Gearmotor alternative: İRAM 53 / 80 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="N66" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=29.85 + IEC 80 B5 input (code 155) | Catalogue ratio i=29.85 (n2≈46 rpm), Sf 3.22 at 0.75 kW; Gearmotor alternative: İRAM 63 / 80 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=29.85 + IEC 80 B5 input (code 155) | Catalogue ratio i=29.85 (n2≈46 rpm), Sf 3.22 at 0.75 kW; Gearmotor alternative: İRAM 63 / 80 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -5458,7 +5458,7 @@
       </c>
       <c r="N67" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 731 i=39.88 + IEC 80 B5 input (code 155) | Catalogue ratio i=39.88 (n2≈35 rpm), Sf 3.22 at 0.75 kW; Gearmotor alternative: İRAM 731 / 80 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 731 i=39.88 + IEC 80 B5 input (code 155) | Catalogue ratio i=39.88 (n2≈35 rpm), Sf 3.22 at 0.75 kW; Gearmotor alternative: İRAM 731 / 80 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="N68" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 52 i=9.47 + IEC 90 B5 input (code 155) | Catalogue ratio i=9.47 (n2≈147 rpm), Sf 2.2 at 1.1 kW; Gearmotor alternative: İRAM 52 / 90 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 52 i=9.47 + IEC 90 B5 input (code 155) | Catalogue ratio i=9.47 (n2≈147 rpm), Sf 2.2 at 1.1 kW; Gearmotor alternative: İRAM 52 / 90 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5586,7 +5586,7 @@
       </c>
       <c r="N69" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 62 i=15.13 + IEC 90 B5 input (code 155) | Catalogue ratio i=15.13 (n2≈92 rpm), Sf 3.75 at 1.1 kW; Gearmotor alternative: İRAM 62 / 90 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 62 i=15.13 + IEC 90 B5 input (code 155) | Catalogue ratio i=15.13 (n2≈92 rpm), Sf 3.75 at 1.1 kW; Gearmotor alternative: İRAM 62 / 90 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5650,7 +5650,7 @@
       </c>
       <c r="N70" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=20.53 + IEC 90 B5 input (code 155) | Catalogue ratio i=20.53 (n2≈68 rpm), Sf 3.2 at 1.1 kW; Gearmotor alternative: İRAM 63 / 90 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=20.53 + IEC 90 B5 input (code 155) | Catalogue ratio i=20.53 (n2≈68 rpm), Sf 3.2 at 1.1 kW; Gearmotor alternative: İRAM 63 / 90 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5714,7 +5714,7 @@
       </c>
       <c r="N71" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=29.85 + IEC 90 B5 input (code 155) | Catalogue ratio i=29.85 (n2≈46 rpm), Sf 2.19 at 1.1 kW; Gearmotor alternative: İRAM 63 / 90 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=29.85 + IEC 90 B5 input (code 155) | Catalogue ratio i=29.85 (n2≈46 rpm), Sf 2.19 at 1.1 kW; Gearmotor alternative: İRAM 63 / 90 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="N72" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 73 i=41.66 + IEC 90 B5 input (code 155) | Catalogue ratio i=41.66 (n2≈33 rpm), Sf 2.79 at 1.1 kW; Gearmotor alternative: İRAM 73 / 90 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 73 i=41.66 + IEC 90 B5 input (code 155) | Catalogue ratio i=41.66 (n2≈33 rpm), Sf 2.79 at 1.1 kW; Gearmotor alternative: İRAM 73 / 90 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5842,7 +5842,7 @@
       </c>
       <c r="N73" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 62 i=10.07 + IEC 90 B5 input (code 155) | Catalogue ratio i=10.07 (n2≈138 rpm), Sf 3.81 at 1.5 kW; Gearmotor alternative: İRAM 62 / 90 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 62 i=10.07 + IEC 90 B5 input (code 155) | Catalogue ratio i=10.07 (n2≈138 rpm), Sf 3.81 at 1.5 kW; Gearmotor alternative: İRAM 62 / 90 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5906,7 @@
       </c>
       <c r="N74" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=20.53 + IEC 90 B5 input (code 155) | Catalogue ratio i=20.53 (n2≈68 rpm), Sf 2.34 at 1.5 kW; Gearmotor alternative: İRAM 63 / 90 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=20.53 + IEC 90 B5 input (code 155) | Catalogue ratio i=20.53 (n2≈68 rpm), Sf 2.34 at 1.5 kW; Gearmotor alternative: İRAM 63 / 90 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="N75" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=29.85 + IEC 90 B5 input (code 155) | Catalogue ratio i=29.85 (n2≈46 rpm), Sf 1.61 at 1.5 kW; Gearmotor alternative: İRAM 63 / 90 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=29.85 + IEC 90 B5 input (code 155) | Catalogue ratio i=29.85 (n2≈46 rpm), Sf 1.61 at 1.5 kW; Gearmotor alternative: İRAM 63 / 90 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="N76" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 73 i=41.66 + IEC 90 B5 input (code 155) | Catalogue ratio i=41.66 (n2≈33 rpm), Sf 2.05 at 1.5 kW; Gearmotor alternative: İRAM 73 / 90 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 73 i=41.66 + IEC 90 B5 input (code 155) | Catalogue ratio i=41.66 (n2≈33 rpm), Sf 2.05 at 1.5 kW; Gearmotor alternative: İRAM 73 / 90 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="N77" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 62 i=10.07 + IEC 100 B5 input (code 155) | Catalogue ratio i=10.07 (n2≈138 rpm), Sf 2.6 at 2.2 kW; Gearmotor alternative: İRAM 62 / 100 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 62 i=10.07 + IEC 100 B5 input (code 155) | Catalogue ratio i=10.07 (n2≈138 rpm), Sf 2.6 at 2.2 kW; Gearmotor alternative: İRAM 62 / 100 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="N78" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=15.59 + IEC 100 B5 input (code 155) | Catalogue ratio i=15.59 (n2≈89 rpm), Sf 2.04 at 2.2 kW; Gearmotor alternative: İRAM 63 / 100 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=15.59 + IEC 100 B5 input (code 155) | Catalogue ratio i=15.59 (n2≈89 rpm), Sf 2.04 at 2.2 kW; Gearmotor alternative: İRAM 63 / 100 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6226,7 +6226,7 @@
       </c>
       <c r="N79" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=20.53 + IEC 100 B5 input (code 155) | Catalogue ratio i=20.53 (n2≈68 rpm), Sf 1.6 at 2.2 kW; Gearmotor alternative: İRAM 63 / 100 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 63 i=20.53 + IEC 100 B5 input (code 155) | Catalogue ratio i=20.53 (n2≈68 rpm), Sf 1.6 at 2.2 kW; Gearmotor alternative: İRAM 63 / 100 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6290,7 +6290,7 @@
       </c>
       <c r="N80" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 73 i=31.16 + IEC 100 B5 input (code 155) | Catalogue ratio i=31.16 (n2≈44 rpm), Sf 1.75 at 2.2 kW; Gearmotor alternative: İRAM 73 / 100 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 73 i=31.16 + IEC 100 B5 input (code 155) | Catalogue ratio i=31.16 (n2≈44 rpm), Sf 1.75 at 2.2 kW; Gearmotor alternative: İRAM 73 / 100 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6354,7 +6354,7 @@
       </c>
       <c r="N81" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 83 i=41.22 + IEC 100 B5 input (code 155) | Catalogue ratio i=41.22 (n2≈33 rpm), Sf 2.45 at 2.2 kW; Gearmotor alternative: İRAM 83 / 100 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRAP 83 i=41.22 + IEC 100 B5 input (code 155) | Catalogue ratio i=41.22 (n2≈33 rpm), Sf 2.45 at 2.2 kW; Gearmotor alternative: İRAM 83 / 100 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="N82" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 62 i=10.07 + IEC 100 B5 input (code 155) | Catalogue ratio i=10.07 (n2≈138 rpm), Sf 1.9 at 3 kW; Gearmotor alternative: İRFM 62 / 100 L 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 62 i=10.07 + IEC 100 B5 input (code 155) | Catalogue ratio i=10.07 (n2≈138 rpm), Sf 1.9 at 3 kW; Gearmotor alternative: İRFM 62 / 100 L 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -6482,7 +6482,7 @@
       </c>
       <c r="N83" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 73 i=20.29 + IEC 100 B5 input (code 155) | Catalogue ratio i=20.29 (n2≈68 rpm), Sf 2.01 at 3 kW; Gearmotor alternative: İRFM 73 / 100 L 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 73 i=20.29 + IEC 100 B5 input (code 155) | Catalogue ratio i=20.29 (n2≈68 rpm), Sf 2.01 at 3 kW; Gearmotor alternative: İRFM 73 / 100 L 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -6546,7 +6546,7 @@
       </c>
       <c r="N84" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=30.08 + IEC 100 B5 input (code 155) | Catalogue ratio i=30.08 (n2≈46 rpm), Sf 2.55 at 3 kW; Gearmotor alternative: İRFM 83 / 100 L 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=30.08 + IEC 100 B5 input (code 155) | Catalogue ratio i=30.08 (n2≈46 rpm), Sf 2.55 at 3 kW; Gearmotor alternative: İRFM 83 / 100 L 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6610,7 @@
       </c>
       <c r="N85" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=41.22 + IEC 100 B5 input (code 155) | Catalogue ratio i=41.22 (n2≈33 rpm), Sf 1.8 at 3 kW; Gearmotor alternative: İRFM 83 / 100 L 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=41.22 + IEC 100 B5 input (code 155) | Catalogue ratio i=41.22 (n2≈33 rpm), Sf 1.8 at 3 kW; Gearmotor alternative: İRFM 83 / 100 L 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="N86" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 721 i=9.866 + IEC 112 B5 input (code 155) | Catalogue ratio i=9.866 (n2≈141 rpm), Sf 1.8 at 4 kW; Gearmotor alternative: İRFM 721 / 112 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 721 i=9.866 + IEC 112 B5 input (code 155) | Catalogue ratio i=9.866 (n2≈141 rpm), Sf 1.8 at 4 kW; Gearmotor alternative: İRFM 721 / 112 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="N87" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 73 i=20.29 + IEC 112 B5 input (code 155) | Catalogue ratio i=20.29 (n2≈68 rpm), Sf 1.51 at 4 kW; Gearmotor alternative: İRFM 73 / 112 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 73 i=20.29 + IEC 112 B5 input (code 155) | Catalogue ratio i=20.29 (n2≈68 rpm), Sf 1.51 at 4 kW; Gearmotor alternative: İRFM 73 / 112 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -6802,7 +6802,7 @@
       </c>
       <c r="N88" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=30.08 + IEC 112 B5 input (code 155) | Catalogue ratio i=30.08 (n2≈46 rpm), Sf 1.91 at 4 kW; Gearmotor alternative: İRFM 83 / 112 M 4b (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=30.08 + IEC 112 B5 input (code 155) | Catalogue ratio i=30.08 (n2≈46 rpm), Sf 1.91 at 4 kW; Gearmotor alternative: İRFM 83 / 112 M 4b (available on request)</t>
         </is>
       </c>
     </row>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="N89" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 82 i=9.689 + IEC 132 B5 input (code 155) | Catalogue ratio i=9.689 (n2≈144 rpm), Sf 3.38 at 5.5 kW; Gearmotor alternative: İRFM 82 / 132 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 82 i=9.689 + IEC 132 B5 input (code 155) | Catalogue ratio i=9.689 (n2≈144 rpm), Sf 3.38 at 5.5 kW; Gearmotor alternative: İRFM 82 / 132 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="N90" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=20.26 + IEC 132 B5 input (code 155) | Catalogue ratio i=20.26 (n2≈69 rpm), Sf 2.0 at 5.5 kW; Gearmotor alternative: İRFM 83 / 132 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 83 i=20.26 + IEC 132 B5 input (code 155) | Catalogue ratio i=20.26 (n2≈69 rpm), Sf 2.0 at 5.5 kW; Gearmotor alternative: İRFM 83 / 132 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -6994,7 +6994,7 @@
       </c>
       <c r="N91" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 93 i=29.52 + IEC 132 B5 input (code 155) | Catalogue ratio i=29.52 (n2≈47 rpm), Sf 2.62 at 5.5 kW; Gearmotor alternative: İRFM 93 / 132 S 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 93 i=29.52 + IEC 132 B5 input (code 155) | Catalogue ratio i=29.52 (n2≈47 rpm), Sf 2.62 at 5.5 kW; Gearmotor alternative: İRFM 93 / 132 S 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="N92" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 82 i=9.689 + IEC 132 B5 input (code 155) | Catalogue ratio i=9.689 (n2≈144 rpm), Sf 2.48 at 7.5 kW; Gearmotor alternative: İRFM 82 / 132 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 82 i=9.689 + IEC 132 B5 input (code 155) | Catalogue ratio i=9.689 (n2≈144 rpm), Sf 2.48 at 7.5 kW; Gearmotor alternative: İRFM 82 / 132 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="N93" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 92 i=20.6 + IEC 132 B5 input (code 155) | Catalogue ratio i=20.6 (n2≈67 rpm), Sf 2.4 at 7.5 kW; Gearmotor alternative: İRFM 92 / 132 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 92 i=20.6 + IEC 132 B5 input (code 155) | Catalogue ratio i=20.6 (n2≈67 rpm), Sf 2.4 at 7.5 kW; Gearmotor alternative: İRFM 92 / 132 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -7186,7 +7186,7 @@
       </c>
       <c r="N94" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 82 i=9.689 + IEC 160 B5 input (code 155) | Catalogue ratio i=9.689 (n2≈144 rpm), Sf 1.69 at 11 kW; Gearmotor alternative: İRFM 82 / 160 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 82 i=9.689 + IEC 160 B5 input (code 155) | Catalogue ratio i=9.689 (n2≈144 rpm), Sf 1.69 at 11 kW; Gearmotor alternative: İRFM 82 / 160 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="N95" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 92 i=20.6 + IEC 160 B5 input (code 155) | Catalogue ratio i=20.6 (n2≈67 rpm), Sf 1.64 at 11 kW; Gearmotor alternative: İRFM 92 / 160 M 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 92 i=20.6 + IEC 160 B5 input (code 155) | Catalogue ratio i=20.6 (n2≈67 rpm), Sf 1.64 at 11 kW; Gearmotor alternative: İRFM 92 / 160 M 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="N96" s="175" t="inlineStr">
         <is>
-          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 103 i=20.31 + IEC 160 B5 input (code 155) | Catalogue ratio i=20.31 (n2≈68 rpm), Sf 2.1 at 15 kW; Gearmotor alternative: İRFM 103 / 160 L 4a (not priced)</t>
+          <t>Quote reducer-only and complete gearmotor alternatives || OFFERED: İ.Mak İRFP 103 i=20.31 + IEC 160 B5 input (code 155) | Catalogue ratio i=20.31 (n2≈68 rpm), Sf 2.1 at 15 kW; Gearmotor alternative: İRFM 103 / 160 L 4a (available on request)</t>
         </is>
       </c>
     </row>
@@ -7378,7 +7378,7 @@
       </c>
       <c r="N97" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 80 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 5.4 at 0.75 kW; Torque arm included in unit price | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 80 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 5.4 at 0.75 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="N98" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 42-TR i=14.25 + IEC 80 B5 | Catalogue ratio i=14.25 (n2≈98 rpm), Sf 2.9 at 0.75 kW; Torque arm included in unit price | Options (list → net): Shrink disc €54.00 → €35.10</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 42-TR i=14.25 + IEC 80 B5 | Catalogue ratio i=14.25 (n2≈98 rpm), Sf 2.9 at 0.75 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €35.10</t>
         </is>
       </c>
     </row>
@@ -7506,7 +7506,7 @@
       </c>
       <c r="N99" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=19.83 + IEC 80 B5 | Catalogue ratio i=19.83 (n2≈71 rpm), Sf 2.7 at 0.75 kW; Torque arm included in unit price | Options (list → net): Shrink disc €54.00 → €35.10</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=19.83 + IEC 80 B5 | Catalogue ratio i=19.83 (n2≈71 rpm), Sf 2.7 at 0.75 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €35.10</t>
         </is>
       </c>
     </row>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="N100" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=29.92 + IEC 80 B5 | Catalogue ratio i=29.92 (n2≈47 rpm), Sf 1.69 at 0.75 kW; Torque arm included in unit price | Options (list → net): Shrink disc €54.00 → €35.10</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=29.92 + IEC 80 B5 | Catalogue ratio i=29.92 (n2≈47 rpm), Sf 1.69 at 0.75 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €35.10</t>
         </is>
       </c>
     </row>
@@ -7634,7 +7634,7 @@
       </c>
       <c r="N101" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 90 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 3.7 at 1.1 kW; Torque arm included in unit price | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 90 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 3.7 at 1.1 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -7698,7 +7698,7 @@
       </c>
       <c r="N102" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=19.83 + IEC 90 B5 | Catalogue ratio i=19.83 (n2≈71 rpm), Sf 1.85 at 1.1 kW; Torque arm included in unit price | Options (list → net): Shrink disc €54.00 → €35.10</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=19.83 + IEC 90 B5 | Catalogue ratio i=19.83 (n2≈71 rpm), Sf 1.85 at 1.1 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €35.10</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
       </c>
       <c r="N103" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=30.93 + IEC 90 B5 | Catalogue ratio i=30.93 (n2≈45 rpm), Sf 1.8 at 1.1 kW; Torque arm included in unit price | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=30.93 + IEC 90 B5 | Catalogue ratio i=30.93 (n2≈45 rpm), Sf 1.8 at 1.1 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="N104" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=42.21 + IEC 90 B5 | Catalogue ratio i=42.21 (n2≈33 rpm), Sf 2.7 at 1.1 kW; Torque arm included in unit price | Options (list → net): Shrink disc €103.00 → €66.95</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=42.21 + IEC 90 B5 | Catalogue ratio i=42.21 (n2≈33 rpm), Sf 2.7 at 1.1 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €66.95</t>
         </is>
       </c>
     </row>
@@ -7890,7 +7890,7 @@
       </c>
       <c r="N105" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 90 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 2.7 at 1.5 kW; Torque arm included in unit price | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 90 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 2.7 at 1.5 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -7954,7 +7954,7 @@
       </c>
       <c r="N106" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=15.73 + IEC 90 B5 | Catalogue ratio i=15.73 (n2≈89 rpm), Sf 1.72 at 1.5 kW; Torque arm included in unit price | Options (list → net): Shrink disc €54.00 → €35.10</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 43-TR i=15.73 + IEC 90 B5 | Catalogue ratio i=15.73 (n2≈89 rpm), Sf 1.72 at 1.5 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €35.10</t>
         </is>
       </c>
     </row>
@@ -8018,7 +8018,7 @@
       </c>
       <c r="N107" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=19.11 + IEC 90 B5 | Catalogue ratio i=19.11 (n2≈73 rpm), Sf 2.0 at 1.5 kW; Torque arm included in unit price | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=19.11 + IEC 90 B5 | Catalogue ratio i=19.11 (n2≈73 rpm), Sf 2.0 at 1.5 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="N108" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=28.39 + IEC 90 B5 | Catalogue ratio i=28.39 (n2≈49 rpm), Sf 2.9 at 1.5 kW; Torque arm included in unit price | Options (list → net): Shrink disc €103.00 → €66.95</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=28.39 + IEC 90 B5 | Catalogue ratio i=28.39 (n2≈49 rpm), Sf 2.9 at 1.5 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €66.95</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="N109" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=42.21 + IEC 90 B5 | Catalogue ratio i=42.21 (n2≈33 rpm), Sf 1.98 at 1.5 kW; Torque arm included in unit price | Options (list → net): Shrink disc €103.00 → €66.95</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=42.21 + IEC 90 B5 | Catalogue ratio i=42.21 (n2≈33 rpm), Sf 1.98 at 1.5 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €66.95</t>
         </is>
       </c>
     </row>
@@ -8210,7 +8210,7 @@
       </c>
       <c r="N110" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 100 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 1.84 at 2.2 kW; Torque arm included in unit price | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=10.44 + IEC 100 B5 | Catalogue ratio i=10.44 (n2≈134 rpm), Sf 1.84 at 2.2 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -8274,7 +8274,7 @@
       </c>
       <c r="N111" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=15.04 + IEC 100 B5 | Catalogue ratio i=15.04 (n2≈93 rpm), Sf 1.64 at 2.2 kW; Torque arm included in unit price | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 63-TR i=15.04 + IEC 100 B5 | Catalogue ratio i=15.04 (n2≈93 rpm), Sf 1.64 at 2.2 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -8338,7 +8338,7 @@
       </c>
       <c r="N112" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=19.51 + IEC 100 B5 | Catalogue ratio i=19.51 (n2≈72 rpm), Sf 2.7 at 2.2 kW; Torque arm included in unit price | Options (list → net): Shrink disc €103.00 → €66.95</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 73-TR i=19.51 + IEC 100 B5 | Catalogue ratio i=19.51 (n2≈72 rpm), Sf 2.7 at 2.2 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €66.95</t>
         </is>
       </c>
     </row>
@@ -8402,7 +8402,7 @@
       </c>
       <c r="N113" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 83-TR i=31.34 + IEC 100 B5 | Catalogue ratio i=31.34 (n2≈45 rpm), Sf 3.3 at 2.2 kW; Torque arm included in unit price | Options (list → net): Shrink disc €162.00 → €105.30</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 83-TR i=31.34 + IEC 100 B5 | Catalogue ratio i=31.34 (n2≈45 rpm), Sf 3.3 at 2.2 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €105.30</t>
         </is>
       </c>
     </row>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="N114" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm || OFFERED: İ.Mak İRKP 83-TR i=37.93 + IEC 100 B5 | Catalogue ratio i=37.93 (n2≈37 rpm), Sf 2.5 at 2.2 kW; Torque arm included in unit price | Options (list → net): Shrink disc €162.00 → €105.30</t>
+          <t>Include torque arm || OFFERED: İ.Mak İRKP 83-TR i=37.93 + IEC 100 B5 | Catalogue ratio i=37.93 (n2≈37 rpm), Sf 2.5 at 2.2 kW; Torque arm included in unit price | Options included in Unit Price: Shrink disc €105.30</t>
         </is>
       </c>
     </row>
@@ -8530,7 +8530,7 @@
       </c>
       <c r="N115" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 73-SR i=15.53 + IEC 100 B5 (foot mounted) | Catalogue ratio i=15.53 (n2≈90 rpm), Sf 2.2 at 3 kW | Options (list → net): Output flange €32.00 → €20.80</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 73-SR i=15.53 + IEC 100 B5 (foot mounted) | Catalogue ratio i=15.53 (n2≈90 rpm), Sf 2.2 at 3 kW | Options included in Unit Price: Output flange €20.80</t>
         </is>
       </c>
     </row>
@@ -8594,7 +8594,7 @@
       </c>
       <c r="N116" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 73-SR i=19.51 + IEC 100 B5 (foot mounted) | Catalogue ratio i=19.51 (n2≈72 rpm), Sf 1.94 at 3 kW | Options (list → net): Output flange €32.00 → €20.80</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 73-SR i=19.51 + IEC 100 B5 (foot mounted) | Catalogue ratio i=19.51 (n2≈72 rpm), Sf 1.94 at 3 kW | Options included in Unit Price: Output flange €20.80</t>
         </is>
       </c>
     </row>
@@ -8658,7 +8658,7 @@
       </c>
       <c r="N117" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=31.34 + IEC 100 B5 (foot mounted) | Catalogue ratio i=31.34 (n2≈45 rpm), Sf 2.4 at 3 kW | Options (list → net): Output flange €40.00 → €26.00</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=31.34 + IEC 100 B5 (foot mounted) | Catalogue ratio i=31.34 (n2≈45 rpm), Sf 2.4 at 3 kW | Options included in Unit Price: Output flange €26.00</t>
         </is>
       </c>
     </row>
@@ -8722,7 +8722,7 @@
       </c>
       <c r="N118" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 73-SR i=15.53 + IEC 112 B5 (foot mounted) | Catalogue ratio i=15.53 (n2≈90 rpm), Sf 1.65 at 4 kW | Options (list → net): Output flange €32.00 → €20.80</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 73-SR i=15.53 + IEC 112 B5 (foot mounted) | Catalogue ratio i=15.53 (n2≈90 rpm), Sf 1.65 at 4 kW | Options included in Unit Price: Output flange €20.80</t>
         </is>
       </c>
     </row>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="N119" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=19.33 + IEC 112 B5 (foot mounted) | Catalogue ratio i=19.33 (n2≈72 rpm), Sf 2.7 at 4 kW | Options (list → net): Output flange €40.00 → €26.00</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=19.33 + IEC 112 B5 (foot mounted) | Catalogue ratio i=19.33 (n2≈72 rpm), Sf 2.7 at 4 kW | Options included in Unit Price: Output flange €26.00</t>
         </is>
       </c>
     </row>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="N120" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=31.34 + IEC 112 B5 (foot mounted) | Catalogue ratio i=31.34 (n2≈45 rpm), Sf 1.81 at 4 kW | Options (list → net): Output flange €40.00 → €26.00</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=31.34 + IEC 112 B5 (foot mounted) | Catalogue ratio i=31.34 (n2≈45 rpm), Sf 1.81 at 4 kW | Options included in Unit Price: Output flange €26.00</t>
         </is>
       </c>
     </row>
@@ -8914,7 +8914,7 @@
       </c>
       <c r="N121" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=19.33 + IEC 132 B5 (foot mounted) | Catalogue ratio i=19.33 (n2≈72 rpm), Sf 2.0 at 5.5 kW | Options (list → net): Output flange €40.00 → €26.00</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 83-SR i=19.33 + IEC 132 B5 (foot mounted) | Catalogue ratio i=19.33 (n2≈72 rpm), Sf 2.0 at 5.5 kW | Options included in Unit Price: Output flange €26.00</t>
         </is>
       </c>
     </row>
@@ -8978,7 +8978,7 @@
       </c>
       <c r="N122" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 93-SR i=29.78 + IEC 132 B5 (foot mounted) | Catalogue ratio i=29.78 (n2≈47 rpm), Sf 2.4 at 5.5 kW | Options (list → net): Output flange €71.00 → €46.15</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 93-SR i=29.78 + IEC 132 B5 (foot mounted) | Catalogue ratio i=29.78 (n2≈47 rpm), Sf 2.4 at 5.5 kW | Options included in Unit Price: Output flange €46.15</t>
         </is>
       </c>
     </row>
@@ -9042,7 +9042,7 @@
       </c>
       <c r="N123" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 93-SR i=20.8 + IEC 132 B5 (foot mounted) | Catalogue ratio i=20.8 (n2≈67 rpm), Sf 2.4 at 7.5 kW | Options (list → net): Output flange €71.00 → €46.15</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 93-SR i=20.8 + IEC 132 B5 (foot mounted) | Catalogue ratio i=20.8 (n2≈67 rpm), Sf 2.4 at 7.5 kW | Options included in Unit Price: Output flange €46.15</t>
         </is>
       </c>
     </row>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="N124" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 103-SR i=30.65 + IEC 160 B5 (foot mounted) | Catalogue ratio i=30.65 (n2≈46 rpm), Sf 1.9 at 11 kW | Options (list → net): Output flange €129.00 → €83.85</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 103-SR i=30.65 + IEC 160 B5 (foot mounted) | Catalogue ratio i=30.65 (n2≈46 rpm), Sf 1.9 at 11 kW | Options included in Unit Price: Output flange €83.85</t>
         </is>
       </c>
     </row>
@@ -9170,7 +9170,7 @@
       </c>
       <c r="N125" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 123-SR i=30.13 + IEC 160 B5 (foot mounted) | Catalogue ratio i=30.13 (n2≈46 rpm), Sf 2.4 at 15 kW | Options (list → net): Output flange €192.00 → €124.80</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 123-SR i=30.13 + IEC 160 B5 (foot mounted) | Catalogue ratio i=30.13 (n2≈46 rpm), Sf 2.4 at 15 kW | Options included in Unit Price: Output flange €124.80</t>
         </is>
       </c>
     </row>
@@ -9234,7 +9234,7 @@
       </c>
       <c r="N126" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak İRKP 143-SR i=41.15 + IEC 180 B5 (foot mounted) | Catalogue ratio i=41.15 (n2≈34 rpm), Sf 2.2 at 22 kW | Options (list → net): Output flange €302.00 → €196.30</t>
+          <t>Quote output flange option || OFFERED: İ.Mak İRKP 143-SR i=41.15 + IEC 180 B5 (foot mounted) | Catalogue ratio i=41.15 (n2≈34 rpm), Sf 2.2 at 22 kW | Options included in Unit Price: Output flange €196.30</t>
         </is>
       </c>
     </row>
@@ -9298,7 +9298,7 @@
       </c>
       <c r="N127" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 52-TL i=9.997 + IEC 90 B5 | Catalogue ratio i=9.997 (n2≈140 rpm), Sf 1.98 at 1.5 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €60.00 → €39.00</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 52-TL i=9.997 + IEC 90 B5 | Catalogue ratio i=9.997 (n2≈140 rpm), Sf 1.98 at 1.5 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €39.00</t>
         </is>
       </c>
     </row>
@@ -9362,7 +9362,7 @@
       </c>
       <c r="N128" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 62-TL i=20.18 + IEC 90 B5 | Catalogue ratio i=20.18 (n2≈69 rpm), Sf 2.1 at 1.5 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 62-TL i=20.18 + IEC 90 B5 | Catalogue ratio i=20.18 (n2≈69 rpm), Sf 2.1 at 1.5 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -9426,7 +9426,7 @@
       </c>
       <c r="N129" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 62-TL i=14.78 + IEC 100 B5 | Catalogue ratio i=14.78 (n2≈95 rpm), Sf 1.85 at 2.2 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €68.00 → €44.20</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 62-TL i=14.78 + IEC 100 B5 | Catalogue ratio i=14.78 (n2≈95 rpm), Sf 1.85 at 2.2 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €44.20</t>
         </is>
       </c>
     </row>
@@ -9490,7 +9490,7 @@
       </c>
       <c r="N130" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 73-TL i=29.69 + IEC 100 B5 | Catalogue ratio i=29.69 (n2≈47 rpm), Sf 1.85 at 2.2 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €103.00 → €66.95</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 73-TL i=29.69 + IEC 100 B5 | Catalogue ratio i=29.69 (n2≈47 rpm), Sf 1.85 at 2.2 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €66.95</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="N131" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 72-TL i=19.89 + IEC 100 B5 | Catalogue ratio i=19.89 (n2≈70 rpm), Sf 2.1 at 3 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €103.00 → €66.95</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 72-TL i=19.89 + IEC 100 B5 | Catalogue ratio i=19.89 (n2≈70 rpm), Sf 2.1 at 3 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €66.95</t>
         </is>
       </c>
     </row>
@@ -9618,7 +9618,7 @@
       </c>
       <c r="N132" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 83-TL i=42.58 + IEC 100 B5 | Catalogue ratio i=42.58 (n2≈33 rpm), Sf 1.85 at 3 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €162.00 → €105.30</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 83-TL i=42.58 + IEC 100 B5 | Catalogue ratio i=42.58 (n2≈33 rpm), Sf 1.85 at 3 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €105.30</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="N133" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 72-TL i=19.89 + IEC 112 B5 | Catalogue ratio i=19.89 (n2≈70 rpm), Sf 1.57 at 4 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €103.00 → €66.95</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 72-TL i=19.89 + IEC 112 B5 | Catalogue ratio i=19.89 (n2≈70 rpm), Sf 1.57 at 4 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €66.95</t>
         </is>
       </c>
     </row>
@@ -9746,7 +9746,7 @@
       </c>
       <c r="N134" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 83-TL i=30.34 + IEC 112 B5 | Catalogue ratio i=30.34 (n2≈46 rpm), Sf 1.95 at 4 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €162.00 → €105.30</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 83-TL i=30.34 + IEC 112 B5 | Catalogue ratio i=30.34 (n2≈46 rpm), Sf 1.95 at 4 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €105.30</t>
         </is>
       </c>
     </row>
@@ -9810,7 +9810,7 @@
       </c>
       <c r="N135" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 82-TL i=20.69 + IEC 132 B5 | Catalogue ratio i=20.69 (n2≈68 rpm), Sf 1.69 at 5.5 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €162.00 → €105.30</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 82-TL i=20.69 + IEC 132 B5 | Catalogue ratio i=20.69 (n2≈68 rpm), Sf 1.69 at 5.5 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €105.30</t>
         </is>
       </c>
     </row>
@@ -9874,7 +9874,7 @@
       </c>
       <c r="N136" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 93-TL i=40.62 + IEC 132 B5 | Catalogue ratio i=40.62 (n2≈34 rpm), Sf 1.92 at 5.5 kW; YP torque arm not in price list – TBC | Options (list → net): Shrink disc €213.00 → €138.45</t>
+          <t>Include torque arm; quote shrink-disc option || OFFERED: İ.Mak YPP 93-TL i=40.62 + IEC 132 B5 | Catalogue ratio i=40.62 (n2≈34 rpm), Sf 1.92 at 5.5 kW; Torque arm: price on request | Options included in Unit Price: Shrink disc €138.45</t>
         </is>
       </c>
     </row>
@@ -9938,7 +9938,7 @@
       </c>
       <c r="N137" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak YPP 92-SL i=26.19 + IEC 132 B5 (foot mounted) | Catalogue ratio i=26.19 (n2≈53 rpm), Sf 2.1 at 7.5 kW | Options (list → net): Output flange €62.00 → €40.30</t>
+          <t>Quote output flange option || OFFERED: İ.Mak YPP 92-SL i=26.19 + IEC 132 B5 (foot mounted) | Catalogue ratio i=26.19 (n2≈53 rpm), Sf 2.1 at 7.5 kW | Options included in Unit Price: Output flange €40.30</t>
         </is>
       </c>
     </row>
@@ -10002,7 +10002,7 @@
       </c>
       <c r="N138" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak YPP 103-SL i=28.84 + IEC 160 B5 (foot mounted) | Catalogue ratio i=28.84 (n2≈49 rpm), Sf 1.94 at 11 kW | Options (list → net): Output flange €115.00 → €74.75</t>
+          <t>Quote output flange option || OFFERED: İ.Mak YPP 103-SL i=28.84 + IEC 160 B5 (foot mounted) | Catalogue ratio i=28.84 (n2≈49 rpm), Sf 1.94 at 11 kW | Options included in Unit Price: Output flange €74.75</t>
         </is>
       </c>
     </row>
@@ -10066,7 +10066,7 @@
       </c>
       <c r="N139" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak YPP 123-SL i=40.73 + IEC 160 B5 (foot mounted) | Catalogue ratio i=40.73 (n2≈34 rpm), Sf 1.83 at 15 kW | Options (list → net): Output flange €174.00 → €113.10</t>
+          <t>Quote output flange option || OFFERED: İ.Mak YPP 123-SL i=40.73 + IEC 160 B5 (foot mounted) | Catalogue ratio i=40.73 (n2≈34 rpm), Sf 1.83 at 15 kW | Options included in Unit Price: Output flange €113.10</t>
         </is>
       </c>
     </row>
@@ -10130,7 +10130,7 @@
       </c>
       <c r="N140" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak YPP 143-SL i=38.8 + IEC 180 B5 (foot mounted) | Catalogue ratio i=38.8 (n2≈36 rpm), Sf 2.4 at 22 kW | Options (list → net): Output flange €275.00 → €178.75</t>
+          <t>Quote output flange option || OFFERED: İ.Mak YPP 143-SL i=38.8 + IEC 180 B5 (foot mounted) | Catalogue ratio i=38.8 (n2≈36 rpm), Sf 2.4 at 22 kW | Options included in Unit Price: Output flange €178.75</t>
         </is>
       </c>
     </row>
@@ -10194,7 +10194,7 @@
       </c>
       <c r="N141" s="175" t="inlineStr">
         <is>
-          <t>Quote output flange option || OFFERED: İ.Mak YPP 153-SL i=50.72 + IEC 200 B5 (foot mounted) | Catalogue ratio i=50.72 (n2≈28 rpm), Sf 1.9 at 30 kW | Options (list → net): Output flange €370.00 → €240.50</t>
+          <t>Quote output flange option || OFFERED: İ.Mak YPP 153-SL i=50.72 + IEC 200 B5 (foot mounted) | Catalogue ratio i=50.72 (n2≈28 rpm), Sf 1.9 at 30 kW | Options included in Unit Price: Output flange €240.50</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="N142" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 01 i=5 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Backstop not available on İRNX 01; Torque arm, pulley and belts – TBC</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 01 i=5 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Backstop not available on İRNX 01; Torque arm, pulley and belts: price on request</t>
         </is>
       </c>
     </row>
@@ -10322,7 +10322,7 @@
       </c>
       <c r="N143" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 01 i=13 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Backstop not available on İRNX 01; Torque arm, pulley and belts – TBC</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 01 i=13 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Backstop not available on İRNX 01; Torque arm, pulley and belts: price on request</t>
         </is>
       </c>
     </row>
@@ -10386,7 +10386,7 @@
       </c>
       <c r="N144" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 01 i=5 + pulley 1:2 (overall ≈1:10) | DEVIATION: input shaft for belt drive, no IEC adaptor available; Overall ratio via pulley 1:2; Backstop not available on İRNX 01; Torque arm, pulley and belts – TBC</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 01 i=5 + pulley 1:2 (overall ≈1:10) | DEVIATION: input shaft for belt drive, no IEC adaptor available; Overall ratio via pulley 1:2; Backstop not available on İRNX 01; Torque arm, pulley and belts: price on request</t>
         </is>
       </c>
     </row>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="N145" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 02 i=20 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts – TBC | Options (list → net): Backstop €149.00 → €96.85</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 02 i=20 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts: price on request | Options included in Unit Price: Backstop €96.85</t>
         </is>
       </c>
     </row>
@@ -10514,7 +10514,7 @@
       </c>
       <c r="N146" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 02 i=13 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts – TBC | Options (list → net): Backstop €149.00 → €96.85</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 02 i=13 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts: price on request | Options included in Unit Price: Backstop €96.85</t>
         </is>
       </c>
     </row>
@@ -10578,7 +10578,7 @@
       </c>
       <c r="N147" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 03 i=21 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts – TBC | Options (list → net): Backstop €149.00 → €96.85</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 03 i=21 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts: price on request | Options included in Unit Price: Backstop €96.85</t>
         </is>
       </c>
     </row>
@@ -10642,7 +10642,7 @@
       </c>
       <c r="N148" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 04 i=20 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts – TBC | Options (list → net): Backstop €197.00 → €128.05</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 04 i=20 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts: price on request | Options included in Unit Price: Backstop €128.05</t>
         </is>
       </c>
     </row>
@@ -10706,7 +10706,7 @@
       </c>
       <c r="N149" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 05 i=21 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts – TBC | Options (list → net): Backstop €197.00 → €128.05</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 05 i=21 | DEVIATION: input shaft for belt drive, no IEC adaptor available; Torque arm, pulley and belts: price on request | Options included in Unit Price: Backstop €128.05</t>
         </is>
       </c>
     </row>
@@ -10770,7 +10770,7 @@
       </c>
       <c r="N150" s="175" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 06 i=13 + pulley 1:2 (overall ≈1:26) | DEVIATION: input shaft for belt drive, no IEC adaptor available; Overall ratio via pulley 1:2; Torque arm, pulley and belts – TBC | Options (list → net): Backstop €245.00 → €159.25</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 06 i=13 + pulley 1:2 (overall ≈1:26) | DEVIATION: input shaft for belt drive, no IEC adaptor available; Overall ratio via pulley 1:2; Torque arm, pulley and belts: price on request | Options included in Unit Price: Backstop €159.25</t>
         </is>
       </c>
     </row>
@@ -10834,7 +10834,7 @@
       </c>
       <c r="N151" s="178" t="inlineStr">
         <is>
-          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 08 i=13 + pulley 1:2 (overall ≈1:26) | DEVIATION: input shaft for belt drive, no IEC adaptor available; Overall ratio via pulley 1:2; Torque arm, pulley and belts – TBC | Options (list → net): Backstop €351.00 → €228.15</t>
+          <t>Include torque arm; quote input shaft, pulley and backstop separately || OFFERED: İ.Mak İRNX 08 i=13 + pulley 1:2 (overall ≈1:26) | DEVIATION: input shaft for belt drive, no IEC adaptor available; Overall ratio via pulley 1:2; Torque arm, pulley and belts: price on request | Options included in Unit Price: Backstop €228.15</t>
         </is>
       </c>
     </row>
@@ -10925,7 +10925,7 @@
       </c>
       <c r="C7" s="181" t="inlineStr">
         <is>
-          <t>TBC – prices based on İ.Mak price list dated 26.01.2026</t>
+          <t>TBC</t>
         </is>
       </c>
     </row>
@@ -10955,7 +10955,7 @@
       </c>
       <c r="C9" s="175" t="inlineStr">
         <is>
-          <t>EXW İ.Mak factory, Turkey. EXW total €216,274.50 net (35% off list, options included), itemised in RFQ Items</t>
+          <t>EXW İ.Mak factory, Turkey. EXW total €216,274.50 (all 145 lines, options included), itemised in RFQ Items</t>
         </is>
       </c>
     </row>
@@ -11195,7 +11195,7 @@
       </c>
       <c r="C25" s="178" t="inlineStr">
         <is>
-          <t>Listed item-by-item in RFQ Items column N (after "||"). Main: GB-046…049 offered as cast-iron İRSA 127 (S series is aluminium); İRNX input shaft only; YP torque arm not in price list</t>
+          <t>Listed item-by-item in RFQ Items column N (after "||"). Main: GB-046…049 offered as cast-iron İRSA 127 (İ.Mak S series is aluminium); İRNX shaft-mounted units have input shaft only (no IEC adaptor); YP torque arm price on request</t>
         </is>
       </c>
     </row>
@@ -11562,7 +11562,7 @@
       <c r="G12" s="184" t="str"/>
       <c r="H12" s="126" t="inlineStr">
         <is>
-          <t>Priced (from price list 26.01.2026)</t>
+          <t>Quoted</t>
         </is>
       </c>
       <c r="I12" s="186" t="n">
@@ -11581,7 +11581,7 @@
       <c r="L12" s="126" t="str"/>
       <c r="M12" s="126" t="inlineStr">
         <is>
-          <t>EUR, 35% off list, options included; see RFQ Items. Large Turkish gearbox manufacturer; strong MENA presence</t>
+          <t>EUR, options included; see RFQ Items. Large Turkish gearbox manufacturer; strong MENA presence</t>
         </is>
       </c>
     </row>

</xml_diff>